<commit_message>
Auto update 2026-06-04 08:22 UTC
</commit_message>
<xml_diff>
--- a/lexus_cars.xlsx
+++ b/lexus_cars.xlsx
@@ -36,7 +36,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -51,6 +51,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -80,12 +85,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -711,9 +719,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y2" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y2" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -814,9 +822,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y3" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y3" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -915,9 +923,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y4" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y4" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -1016,9 +1024,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y5" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y5" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -1119,9 +1127,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y6" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y6" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -1226,9 +1234,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y7" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y7" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -1333,9 +1341,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y8" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y8" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -1436,9 +1444,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y9" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y9" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -1533,9 +1541,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y10" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y10" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -1638,9 +1646,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y11" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y11" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -1749,9 +1757,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y12" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y12" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -1856,9 +1864,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y13" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y13" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -1959,9 +1967,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y14" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y14" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -2064,9 +2072,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y15" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y15" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -2171,9 +2179,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y16" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y16" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -2272,9 +2280,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y17" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y17" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -2373,9 +2381,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y18" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y18" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -2474,9 +2482,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y19" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y19" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -2581,9 +2589,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y20" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y20" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -2686,9 +2694,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y21" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y21" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -2797,9 +2805,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y22" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y22" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -2904,9 +2912,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y23" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y23" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -3001,9 +3009,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y24" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y24" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -3112,9 +3120,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y25" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y25" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -3219,9 +3227,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y26" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y26" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -3322,9 +3330,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y27" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y27" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -3419,9 +3427,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y28" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y28" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -3518,9 +3526,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y29" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y29" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -3625,9 +3633,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y30" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y30" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -3728,9 +3736,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y31" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y31" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -3835,9 +3843,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y32" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y32" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -3942,9 +3950,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y33" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y33" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -4047,9 +4055,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y34" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y34" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -4154,9 +4162,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y35" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y35" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -4255,9 +4263,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y36" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y36" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -4356,9 +4364,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y37" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y37" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -4457,9 +4465,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y38" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y38" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -4558,9 +4566,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y39" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y39" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -4661,9 +4669,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y40" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y40" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -4762,9 +4770,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y41" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y41" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -4863,9 +4871,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y42" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y42" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -4964,9 +4972,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y43" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y43" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -5069,9 +5077,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y44" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y44" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -5174,9 +5182,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y45" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y45" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -5275,9 +5283,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y46" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y46" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -5382,9 +5390,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y47" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y47" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -5489,9 +5497,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y48" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y48" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -5600,9 +5608,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y49" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y49" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -5703,9 +5711,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y50" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y50" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -5804,9 +5812,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y51" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y51" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -5909,9 +5917,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y52" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y52" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -6012,9 +6020,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y53" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y53" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -6113,9 +6121,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y54" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y54" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -6206,9 +6214,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y55" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y55" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update 2026-06-04 08:25 UTC
</commit_message>
<xml_diff>
--- a/lexus_cars.xlsx
+++ b/lexus_cars.xlsx
@@ -36,7 +36,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -56,6 +56,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -85,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -94,6 +99,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -486,8 +494,8 @@
     <col width="40" customWidth="1" min="20" max="20"/>
     <col width="40" customWidth="1" min="21" max="21"/>
     <col width="20" customWidth="1" min="22" max="22"/>
-    <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
     <col width="12" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
@@ -719,9 +727,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y2" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y2" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -822,9 +830,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y3" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y3" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -923,9 +931,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y4" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y4" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -1024,9 +1032,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y5" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y5" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -1127,9 +1135,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y6" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y6" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -1234,9 +1242,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y7" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y7" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -1341,9 +1349,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y8" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y8" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -1444,9 +1452,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y9" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y9" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -1541,9 +1549,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y10" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y10" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -1646,9 +1654,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y11" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y11" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -1757,9 +1765,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y12" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y12" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -1864,9 +1872,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y13" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y13" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -1967,9 +1975,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y14" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y14" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -2072,9 +2080,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y15" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y15" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -2179,9 +2187,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y16" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y16" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -2280,9 +2288,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y17" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y17" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -2381,9 +2389,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y18" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y18" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -2482,9 +2490,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y19" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y19" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -2589,9 +2597,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y20" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y20" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -2694,9 +2702,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y21" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y21" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -2805,9 +2813,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y22" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y22" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -2912,9 +2920,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y23" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y23" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -3009,9 +3017,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y24" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y24" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -3120,9 +3128,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y25" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y25" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -3227,9 +3235,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y26" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y26" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -3330,9 +3338,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y27" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y27" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -3427,9 +3435,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y28" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y28" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -3526,9 +3534,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y29" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y29" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -3633,9 +3641,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y30" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y30" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -3736,9 +3744,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y31" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y31" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -3843,9 +3851,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y32" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y32" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -3950,9 +3958,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y33" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y33" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -4055,9 +4063,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y34" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y34" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -4162,9 +4170,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y35" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y35" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -4263,9 +4271,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y36" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y36" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -4364,9 +4372,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y37" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y37" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -4465,9 +4473,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y38" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y38" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -4566,9 +4574,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y39" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y39" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -4669,9 +4677,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y40" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y40" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -4770,9 +4778,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y41" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y41" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -4871,9 +4879,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y42" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y42" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -4972,9 +4980,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y43" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y43" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -5077,9 +5085,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y44" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y44" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -5182,9 +5190,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y45" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y45" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -5283,9 +5291,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y46" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y46" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -5390,9 +5398,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y47" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y47" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -5497,9 +5505,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y48" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y48" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -5608,9 +5616,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y49" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y49" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -5711,9 +5719,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y50" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y50" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -5812,9 +5820,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y51" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y51" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -5917,9 +5925,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y52" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y52" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -6020,9 +6028,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y53" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y53" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -6121,9 +6129,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y54" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y54" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -6214,9 +6222,9 @@
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="Y55" s="3" t="inlineStr">
-        <is>
-          <t>حذف شده</t>
+      <c r="Y55" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update 2026-06-05 08:58 UTC
</commit_message>
<xml_diff>
--- a/lexus_cars.xlsx
+++ b/lexus_cars.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y55"/>
+  <dimension ref="A1:Y58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5395,12 +5395,12 @@
       </c>
       <c r="X47" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="Y47" s="4" t="inlineStr">
-        <is>
-          <t>بدون تغییر</t>
+          <t>2026-06-05 08:58</t>
+        </is>
+      </c>
+      <c r="Y47" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -5502,12 +5502,12 @@
       </c>
       <c r="X48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="Y48" s="4" t="inlineStr">
-        <is>
-          <t>بدون تغییر</t>
+          <t>2026-06-05 08:58</t>
+        </is>
+      </c>
+      <c r="Y48" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -6225,6 +6225,327 @@
       <c r="Y55" s="4" t="inlineStr">
         <is>
           <t>بدون تغییر</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="40" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>AutoScout24</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Lexus NX</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>NX 300</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>E-Four Luxury Line</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>10/2016</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>161.411 km</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Weiß</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Elektro/Benzin</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>Automatik</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="n">
+        <v>22999</v>
+      </c>
+      <c r="L56" s="2" t="inlineStr"/>
+      <c r="M56" s="2" t="inlineStr"/>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>Erhöhter Preis</t>
+        </is>
+      </c>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="Q56" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="R56" s="2" t="inlineStr">
+        <is>
+          <t>Brühl</t>
+        </is>
+      </c>
+      <c r="S56" s="2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="T56" s="2" t="inlineStr"/>
+      <c r="U56" s="2" t="inlineStr"/>
+      <c r="V56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.autoscout24.de/angebote/lexus-nx-300-e-four-luxury-line-elektro-benzin-weiss-cat_ma43mo20491-5a7fd1aa-8718-4d55-9c8f-d05d41476f85</t>
+        </is>
+      </c>
+      <c r="W56" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 08:58</t>
+        </is>
+      </c>
+      <c r="X56" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 08:58</t>
+        </is>
+      </c>
+      <c r="Y56" s="2" t="inlineStr">
+        <is>
+          <t>جدید</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="40" customHeight="1">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>AutoScout24</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Lexus NX</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>NX 300</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>h Amazing Edition*LED*SHZ*PDC*</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>07/2020</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>61.666 km</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>Schwarz</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>Elektro/Benzin</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>Automatik</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="n">
+        <v>29900</v>
+      </c>
+      <c r="L57" s="2" t="inlineStr"/>
+      <c r="M57" s="2" t="inlineStr"/>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
+          <t>Fairer Preis</t>
+        </is>
+      </c>
+      <c r="O57" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="P57" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="Q57" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="R57" s="2" t="inlineStr">
+        <is>
+          <t>Lohne (Old)</t>
+        </is>
+      </c>
+      <c r="S57" s="2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="T57" s="2" t="inlineStr"/>
+      <c r="U57" s="2" t="inlineStr"/>
+      <c r="V57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.autoscout24.de/angebote/lexus-nx-300-h-amazing-edition-led-shz-pdc-elektro-benzin-schwarz-cat_ma43mo20491-0cfd8fbb-9e23-46c3-b0eb-7f66431071a3</t>
+        </is>
+      </c>
+      <c r="W57" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 08:58</t>
+        </is>
+      </c>
+      <c r="X57" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 08:58</t>
+        </is>
+      </c>
+      <c r="Y57" s="2" t="inlineStr">
+        <is>
+          <t>جدید</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="40" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>AutoScout24</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Lexus NX</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>NX 300</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>h Amazing Edition*LED*SHZ*PDC*</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>07/2020</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>61.666 km</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>Schwarz</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>Benzin</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>Automatik</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="n">
+        <v>29900</v>
+      </c>
+      <c r="L58" s="2" t="inlineStr"/>
+      <c r="M58" s="2" t="inlineStr"/>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>Fairer Preis</t>
+        </is>
+      </c>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="Q58" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="R58" s="2" t="inlineStr">
+        <is>
+          <t>Lohne (Old)</t>
+        </is>
+      </c>
+      <c r="S58" s="2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="T58" s="2" t="inlineStr"/>
+      <c r="U58" s="2" t="inlineStr"/>
+      <c r="V58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.autoscout24.de/angebote/lexus-nx-300-h-amazing-edition-led-shz-pdc-benzin-schwarz-cat_ma43mo20491-0008a11d-96cb-41d1-8435-a0e459ac8472</t>
+        </is>
+      </c>
+      <c r="W58" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 08:58</t>
+        </is>
+      </c>
+      <c r="X58" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 08:58</t>
+        </is>
+      </c>
+      <c r="Y58" s="2" t="inlineStr">
+        <is>
+          <t>جدید</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update 2026-06-06 08:11 UTC
</commit_message>
<xml_diff>
--- a/lexus_cars.xlsx
+++ b/lexus_cars.xlsx
@@ -36,7 +36,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -61,6 +61,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -90,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -102,6 +107,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -469,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y58"/>
+  <dimension ref="A1:Y59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -938,103 +946,107 @@
       </c>
     </row>
     <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>AutoScout24</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Lexus RX</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>RX 450h</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>4WD Comfort Line Trekhaak | 2000 kg trekgewicht |</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>2016</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>01/2016</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>149.662 km</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>Grau</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>Elektro/Benzin</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>Automatik</t>
         </is>
       </c>
-      <c r="K5" s="2" t="n">
+      <c r="K5" s="5" t="n">
+        <v>21995</v>
+      </c>
+      <c r="L5" s="5" t="n">
         <v>20995</v>
       </c>
-      <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="inlineStr"/>
-      <c r="N5" s="2" t="inlineStr"/>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="M5" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="N5" s="5" t="inlineStr"/>
+      <c r="O5" s="5" t="inlineStr">
         <is>
           <t>Nein</t>
         </is>
       </c>
-      <c r="P5" s="2" t="inlineStr">
+      <c r="P5" s="5" t="inlineStr">
         <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="Q5" s="2" t="inlineStr"/>
-      <c r="R5" s="2" t="inlineStr">
+      <c r="Q5" s="5" t="inlineStr"/>
+      <c r="R5" s="5" t="inlineStr">
         <is>
           <t>VEGHEL</t>
         </is>
       </c>
-      <c r="S5" s="2" t="inlineStr">
+      <c r="S5" s="5" t="inlineStr">
         <is>
           <t>NL</t>
         </is>
       </c>
-      <c r="T5" s="2" t="inlineStr"/>
-      <c r="U5" s="2" t="inlineStr"/>
-      <c r="V5" s="2" t="inlineStr">
+      <c r="T5" s="5" t="inlineStr"/>
+      <c r="U5" s="5" t="inlineStr"/>
+      <c r="V5" s="5" t="inlineStr">
         <is>
           <t>https://www.autoscout24.de/angebote/lexus-rx-450h-4wd-comfort-line-trekhaak-2000-kg-trekgewicht-elektro-benzin-grau-cat_ma43mo19238-aa92faff-5996-4d4b-bb11-394c751a1fd4</t>
         </is>
       </c>
-      <c r="W5" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="X5" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="Y5" s="4" t="inlineStr">
-        <is>
-          <t>بدون تغییر</t>
+      <c r="W5" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="X5" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-06 08:11</t>
+        </is>
+      </c>
+      <c r="Y5" s="5" t="inlineStr">
+        <is>
+          <t>تغییر قیمت</t>
         </is>
       </c>
     </row>
@@ -2396,103 +2408,107 @@
       </c>
     </row>
     <row r="19" ht="40" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>AutoScout24</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Lexus RX</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>RX 450h</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>RX 450h 3.5 V6 313 E-Four F SPORT E-CVT</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>2016</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>02/2016</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>175.000 km</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>Schwarz</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="I19" s="5" t="inlineStr">
         <is>
           <t>Benzin</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="J19" s="5" t="inlineStr">
         <is>
           <t>Automatik</t>
         </is>
       </c>
-      <c r="K19" s="2" t="n">
+      <c r="K19" s="5" t="n">
+        <v>25500</v>
+      </c>
+      <c r="L19" s="5" t="n">
         <v>25700</v>
       </c>
-      <c r="L19" s="2" t="inlineStr"/>
-      <c r="M19" s="2" t="inlineStr"/>
-      <c r="N19" s="2" t="inlineStr"/>
-      <c r="O19" s="2" t="inlineStr">
+      <c r="M19" s="5" t="n">
+        <v>-200</v>
+      </c>
+      <c r="N19" s="5" t="inlineStr"/>
+      <c r="O19" s="5" t="inlineStr">
         <is>
           <t>Nein</t>
         </is>
       </c>
-      <c r="P19" s="2" t="inlineStr">
+      <c r="P19" s="5" t="inlineStr">
         <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="Q19" s="2" t="inlineStr"/>
-      <c r="R19" s="2" t="inlineStr">
+      <c r="Q19" s="5" t="inlineStr"/>
+      <c r="R19" s="5" t="inlineStr">
         <is>
           <t>Ivry-sur-Seine</t>
         </is>
       </c>
-      <c r="S19" s="2" t="inlineStr">
+      <c r="S19" s="5" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="T19" s="2" t="inlineStr"/>
-      <c r="U19" s="2" t="inlineStr"/>
-      <c r="V19" s="2" t="inlineStr">
+      <c r="T19" s="5" t="inlineStr"/>
+      <c r="U19" s="5" t="inlineStr"/>
+      <c r="V19" s="5" t="inlineStr">
         <is>
           <t>https://www.autoscout24.de/angebote/lexus-rx-450h-rx-450h-3-5-v6-313-e-four-f-sport-e-cvt-benzin-schwarz-cat_ma43mo19238-e80fa651-625f-43f9-9108-79e132556516</t>
         </is>
       </c>
-      <c r="W19" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="X19" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="Y19" s="4" t="inlineStr">
-        <is>
-          <t>بدون تغییر</t>
+      <c r="W19" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="X19" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-06 08:11</t>
+        </is>
+      </c>
+      <c r="Y19" s="5" t="inlineStr">
+        <is>
+          <t>تغییر قیمت</t>
         </is>
       </c>
     </row>
@@ -6329,9 +6345,9 @@
           <t>2026-06-05 08:58</t>
         </is>
       </c>
-      <c r="Y56" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y56" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -6436,9 +6452,9 @@
           <t>2026-06-05 08:58</t>
         </is>
       </c>
-      <c r="Y57" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y57" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -6543,7 +6559,114 @@
           <t>2026-06-05 08:58</t>
         </is>
       </c>
-      <c r="Y58" s="2" t="inlineStr">
+      <c r="Y58" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="40" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>AutoScout24</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Lexus RX</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>RX 450h</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Luxury RX 450h HEV</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>07/2018</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>80.000 km</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>Schwarz</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>Elektro/Benzin</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>Automatik</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="n">
+        <v>29900</v>
+      </c>
+      <c r="L59" s="2" t="inlineStr"/>
+      <c r="M59" s="2" t="inlineStr"/>
+      <c r="N59" s="2" t="inlineStr"/>
+      <c r="O59" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="P59" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="Q59" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="R59" s="2" t="inlineStr">
+        <is>
+          <t>San Nicolò -  Pc</t>
+        </is>
+      </c>
+      <c r="S59" s="2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="T59" s="2" t="inlineStr">
+        <is>
+          <t>POSSIBILITA' DI FINANZIAMENTO IN SEDE</t>
+        </is>
+      </c>
+      <c r="U59" s="2" t="inlineStr"/>
+      <c r="V59" s="2" t="inlineStr">
+        <is>
+          <t>https://www.autoscout24.de/angebote/lexus-rx-450h-luxury-rx-450h-hev-elektro-benzin-schwarz-cat_ma43mo19238-4a2cf075-6b30-44b2-901d-8e173a5bf142</t>
+        </is>
+      </c>
+      <c r="W59" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-06 08:11</t>
+        </is>
+      </c>
+      <c r="X59" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-06 08:11</t>
+        </is>
+      </c>
+      <c r="Y59" s="2" t="inlineStr">
         <is>
           <t>جدید</t>
         </is>

</xml_diff>

<commit_message>
Auto update 2026-06-07 08:39 UTC
</commit_message>
<xml_diff>
--- a/lexus_cars.xlsx
+++ b/lexus_cars.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y59"/>
+  <dimension ref="A1:Y60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1044,9 +1044,9 @@
           <t>2026-06-06 08:11</t>
         </is>
       </c>
-      <c r="Y5" s="5" t="inlineStr">
-        <is>
-          <t>تغییر قیمت</t>
+      <c r="Y5" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -1663,12 +1663,12 @@
       </c>
       <c r="X11" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="Y11" s="4" t="inlineStr">
-        <is>
-          <t>بدون تغییر</t>
+          <t>2026-06-07 08:39</t>
+        </is>
+      </c>
+      <c r="Y11" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -1774,12 +1774,12 @@
       </c>
       <c r="X12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="Y12" s="4" t="inlineStr">
-        <is>
-          <t>بدون تغییر</t>
+          <t>2026-06-07 08:39</t>
+        </is>
+      </c>
+      <c r="Y12" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -2398,12 +2398,12 @@
       </c>
       <c r="X18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="Y18" s="4" t="inlineStr">
-        <is>
-          <t>بدون تغییر</t>
+          <t>2026-06-07 08:39</t>
+        </is>
+      </c>
+      <c r="Y18" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -2506,9 +2506,9 @@
           <t>2026-06-06 08:11</t>
         </is>
       </c>
-      <c r="Y19" s="5" t="inlineStr">
-        <is>
-          <t>تغییر قیمت</t>
+      <c r="Y19" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,112 @@
           <t>2026-06-06 08:11</t>
         </is>
       </c>
-      <c r="Y59" s="2" t="inlineStr">
+      <c r="Y59" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="40" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>AutoScout24</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Lexus RX</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>RX 450h</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>450h 4WD 3.5 V6 - BV E-CVT 450H</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>04/2016</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>143.000 km</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>Weiß</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>Elektro/Benzin</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>Automatik</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="n">
+        <v>23500</v>
+      </c>
+      <c r="L60" s="2" t="inlineStr"/>
+      <c r="M60" s="2" t="inlineStr"/>
+      <c r="N60" s="2" t="inlineStr"/>
+      <c r="O60" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="P60" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="Q60" s="2" t="inlineStr"/>
+      <c r="R60" s="2" t="inlineStr">
+        <is>
+          <t>Saint-André-de-Corcy</t>
+        </is>
+      </c>
+      <c r="S60" s="2" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="T60" s="2" t="inlineStr">
+        <is>
+          <t>Isofix, Head-up display, 3-Zonen-Klimaautomatik</t>
+        </is>
+      </c>
+      <c r="U60" s="2" t="inlineStr"/>
+      <c r="V60" s="2" t="inlineStr">
+        <is>
+          <t>https://www.autoscout24.de/angebote/lexus-rx-450h-450h-4wd-3-5-v6-bv-e-cvt-450h-elektro-benzin-weiss-cat_ma43mo19238-9c61ccda-f519-46eb-a4fd-cc0b41957bb0</t>
+        </is>
+      </c>
+      <c r="W60" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-07 08:39</t>
+        </is>
+      </c>
+      <c r="X60" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-07 08:39</t>
+        </is>
+      </c>
+      <c r="Y60" s="2" t="inlineStr">
         <is>
           <t>جدید</t>
         </is>

</xml_diff>

<commit_message>
Auto update 2026-06-08 10:08 UTC
</commit_message>
<xml_diff>
--- a/lexus_cars.xlsx
+++ b/lexus_cars.xlsx
@@ -6771,9 +6771,9 @@
           <t>2026-06-07 08:39</t>
         </is>
       </c>
-      <c r="Y60" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+      <c r="Y60" s="4" t="inlineStr">
+        <is>
+          <t>بدون تغییر</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update 2026-06-09 08:50 UTC
</commit_message>
<xml_diff>
--- a/lexus_cars.xlsx
+++ b/lexus_cars.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y60"/>
+  <dimension ref="A1:Y62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3351,12 +3351,12 @@
       </c>
       <c r="X27" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="Y27" s="4" t="inlineStr">
-        <is>
-          <t>بدون تغییر</t>
+          <t>2026-06-09 08:50</t>
+        </is>
+      </c>
+      <c r="Y27" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -6774,6 +6774,216 @@
       <c r="Y60" s="4" t="inlineStr">
         <is>
           <t>بدون تغییر</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="40" customHeight="1">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>AutoScout24</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Lexus RX</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>RX 450h</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>RX450H E-four Privilege !! Vermittlungsverkauf !!</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>02/2019</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>276.930 km</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>Grau</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>Elektro/Benzin</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>Automatik</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="n">
+        <v>26977</v>
+      </c>
+      <c r="L61" s="2" t="inlineStr"/>
+      <c r="M61" s="2" t="inlineStr"/>
+      <c r="N61" s="2" t="inlineStr"/>
+      <c r="O61" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="P61" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="Q61" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="R61" s="2" t="inlineStr">
+        <is>
+          <t>Micheldorf</t>
+        </is>
+      </c>
+      <c r="S61" s="2" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="T61" s="2" t="inlineStr"/>
+      <c r="U61" s="2" t="inlineStr"/>
+      <c r="V61" s="2" t="inlineStr">
+        <is>
+          <t>https://www.autoscout24.de/angebote/lexus-rx-450h-rx450h-e-four-privilege-vermittlungsverkauf-elektro-benzin-grau-cat_ma43mo19238-98466951-0964-433f-a596-e8cb845e2b81</t>
+        </is>
+      </c>
+      <c r="W61" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 08:50</t>
+        </is>
+      </c>
+      <c r="X61" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 08:50</t>
+        </is>
+      </c>
+      <c r="Y61" s="2" t="inlineStr">
+        <is>
+          <t>جدید</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="40" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>AutoScout24</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Lexus NX</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>NX 300h</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>NX 300h Style Edition Aut.*NAV*LED*ACC*CAM*PDC*</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>07/2021</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>64.419 km</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>Grün</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>Elektro/Benzin</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>Automatik</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="n">
+        <v>29170</v>
+      </c>
+      <c r="L62" s="2" t="inlineStr"/>
+      <c r="M62" s="2" t="inlineStr"/>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>Fairer Preis</t>
+        </is>
+      </c>
+      <c r="O62" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="P62" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="Q62" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="R62" s="2" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="S62" s="2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="T62" s="2" t="inlineStr"/>
+      <c r="U62" s="2" t="inlineStr"/>
+      <c r="V62" s="2" t="inlineStr">
+        <is>
+          <t>https://www.autoscout24.de/angebote/lexus-nx-300h-nx-300h-style-edition-aut-nav-led-acc-cam-pdc-elektro-benzin-gruen-cat_ma43mo75908-a079ba42-bc70-4195-9d58-ccb6ca018835</t>
+        </is>
+      </c>
+      <c r="W62" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 08:50</t>
+        </is>
+      </c>
+      <c r="X62" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 08:50</t>
+        </is>
+      </c>
+      <c r="Y62" s="2" t="inlineStr">
+        <is>
+          <t>جدید</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update 2026-06-10 09:07 UTC
</commit_message>
<xml_diff>
--- a/lexus_cars.xlsx
+++ b/lexus_cars.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y62"/>
+  <dimension ref="A1:Y63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3864,12 +3864,12 @@
       </c>
       <c r="X32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="Y32" s="4" t="inlineStr">
-        <is>
-          <t>بدون تغییر</t>
+          <t>2026-06-10 09:07</t>
+        </is>
+      </c>
+      <c r="Y32" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -4284,12 +4284,12 @@
       </c>
       <c r="X36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="Y36" s="4" t="inlineStr">
-        <is>
-          <t>بدون تغییر</t>
+          <t>2026-06-10 09:07</t>
+        </is>
+      </c>
+      <c r="Y36" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -6871,12 +6871,12 @@
       </c>
       <c r="X61" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09 08:50</t>
-        </is>
-      </c>
-      <c r="Y61" s="2" t="inlineStr">
-        <is>
-          <t>جدید</t>
+          <t>2026-06-10 09:07</t>
+        </is>
+      </c>
+      <c r="Y61" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -6978,10 +6978,113 @@
       </c>
       <c r="X62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09 08:50</t>
-        </is>
-      </c>
-      <c r="Y62" s="2" t="inlineStr">
+          <t>2026-06-10 09:07</t>
+        </is>
+      </c>
+      <c r="Y62" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="40" customHeight="1">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>AutoScout24</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Lexus RX</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>RX 450h</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>RX450H E-four Privilege !! Vermittlungsverkauf !!</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>02/2019</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>276.930 km</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>Grau</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>Elektro/Benzin</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>Automatik</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="n">
+        <v>26977</v>
+      </c>
+      <c r="L63" s="2" t="inlineStr"/>
+      <c r="M63" s="2" t="inlineStr"/>
+      <c r="N63" s="2" t="inlineStr"/>
+      <c r="O63" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="P63" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="Q63" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="R63" s="2" t="inlineStr">
+        <is>
+          <t>Micheldorf</t>
+        </is>
+      </c>
+      <c r="S63" s="2" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="T63" s="2" t="inlineStr"/>
+      <c r="U63" s="2" t="inlineStr"/>
+      <c r="V63" s="2" t="inlineStr">
+        <is>
+          <t>https://www.autoscout24.de/angebote/lexus-rx-450h-rx450h-e-four-privilege-vermittlungsverkauf-elektro-benzin-grau-cat_ma43mo19238-058aa86d-c49d-454a-b73e-e77c27094a74</t>
+        </is>
+      </c>
+      <c r="W63" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 09:07</t>
+        </is>
+      </c>
+      <c r="X63" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 09:07</t>
+        </is>
+      </c>
+      <c r="Y63" s="2" t="inlineStr">
         <is>
           <t>جدید</t>
         </is>

</xml_diff>

<commit_message>
Auto update 2026-06-11 09:54 UTC
</commit_message>
<xml_diff>
--- a/lexus_cars.xlsx
+++ b/lexus_cars.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y63"/>
+  <dimension ref="A1:Y67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -732,12 +732,12 @@
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="Y2" s="4" t="inlineStr">
-        <is>
-          <t>بدون تغییر</t>
+          <t>2026-06-11 09:54</t>
+        </is>
+      </c>
+      <c r="Y2" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -2943,99 +2943,103 @@
       </c>
     </row>
     <row r="24" ht="40" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>AutoScout24</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>Lexus RX</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>RX 300</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr"/>
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>2016</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>04/2016</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G24" s="5" t="inlineStr">
         <is>
           <t>85.400 km</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="H24" s="5" t="inlineStr">
         <is>
           <t>Weiß</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="I24" s="5" t="inlineStr">
         <is>
           <t>Benzin</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="J24" s="5" t="inlineStr">
         <is>
           <t>Automatik</t>
         </is>
       </c>
-      <c r="K24" s="2" t="n">
+      <c r="K24" s="5" t="n">
+        <v>23990</v>
+      </c>
+      <c r="L24" s="5" t="n">
         <v>26500</v>
       </c>
-      <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="inlineStr"/>
-      <c r="N24" s="2" t="inlineStr"/>
-      <c r="O24" s="2" t="inlineStr">
+      <c r="M24" s="5" t="n">
+        <v>-2510</v>
+      </c>
+      <c r="N24" s="5" t="inlineStr"/>
+      <c r="O24" s="5" t="inlineStr">
         <is>
           <t>Nein</t>
         </is>
       </c>
-      <c r="P24" s="2" t="inlineStr">
+      <c r="P24" s="5" t="inlineStr">
         <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="2" t="inlineStr">
+      <c r="Q24" s="5" t="inlineStr"/>
+      <c r="R24" s="5" t="inlineStr">
         <is>
           <t>MIJAS</t>
         </is>
       </c>
-      <c r="S24" s="2" t="inlineStr">
+      <c r="S24" s="5" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="T24" s="2" t="inlineStr"/>
-      <c r="U24" s="2" t="inlineStr"/>
-      <c r="V24" s="2" t="inlineStr">
+      <c r="T24" s="5" t="inlineStr"/>
+      <c r="U24" s="5" t="inlineStr"/>
+      <c r="V24" s="5" t="inlineStr">
         <is>
           <t>https://www.autoscout24.de/angebote/lexus-rx-300-benzin-weiss-cat_ma43mo16404-554520c6-0801-4354-b149-54a7a55f738e</t>
         </is>
       </c>
-      <c r="W24" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="X24" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="Y24" s="4" t="inlineStr">
-        <is>
-          <t>بدون تغییر</t>
+      <c r="W24" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="X24" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-11 09:54</t>
+        </is>
+      </c>
+      <c r="Y24" s="5" t="inlineStr">
+        <is>
+          <t>تغییر قیمت</t>
         </is>
       </c>
     </row>
@@ -4076,12 +4080,12 @@
       </c>
       <c r="X34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="Y34" s="4" t="inlineStr">
-        <is>
-          <t>بدون تغییر</t>
+          <t>2026-06-11 09:54</t>
+        </is>
+      </c>
+      <c r="Y34" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
         </is>
       </c>
     </row>
@@ -7081,10 +7085,426 @@
       </c>
       <c r="X63" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10 09:07</t>
-        </is>
-      </c>
-      <c r="Y63" s="2" t="inlineStr">
+          <t>2026-06-11 09:54</t>
+        </is>
+      </c>
+      <c r="Y63" s="3" t="inlineStr">
+        <is>
+          <t>حذف شده</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="40" customHeight="1">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>AutoScout24</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Lexus RX</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>RX 450h</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>RX 450h 3.5i V6 Executive Line E-CVT</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>07/2016</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>215.568 km</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>Silber</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>Elektro/Benzin</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>Automatik</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="n">
+        <v>24900</v>
+      </c>
+      <c r="L64" s="2" t="inlineStr"/>
+      <c r="M64" s="2" t="inlineStr"/>
+      <c r="N64" s="2" t="inlineStr"/>
+      <c r="O64" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="P64" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="Q64" s="2" t="inlineStr"/>
+      <c r="R64" s="2" t="inlineStr">
+        <is>
+          <t>Itterbeek</t>
+        </is>
+      </c>
+      <c r="S64" s="2" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="T64" s="2" t="inlineStr"/>
+      <c r="U64" s="2" t="inlineStr"/>
+      <c r="V64" s="2" t="inlineStr">
+        <is>
+          <t>https://www.autoscout24.de/angebote/lexus-rx-450h-rx-450h-3-5i-v6-executive-line-e-cvt-elektro-benzin-silber-cat_ma43mo19238-a039dde5-c69d-40e0-aa4b-c32fabb59895</t>
+        </is>
+      </c>
+      <c r="W64" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 09:54</t>
+        </is>
+      </c>
+      <c r="X64" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 09:54</t>
+        </is>
+      </c>
+      <c r="Y64" s="2" t="inlineStr">
+        <is>
+          <t>جدید</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="40" customHeight="1">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>AutoScout24</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Lexus NX</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>NX 300</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>300h E-FOUR Launch Edition</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>06/2018</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>58.167 km</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>Silber</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>Elektro/Benzin</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>Automatik</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="n">
+        <v>26440</v>
+      </c>
+      <c r="L65" s="2" t="inlineStr"/>
+      <c r="M65" s="2" t="inlineStr"/>
+      <c r="N65" s="2" t="inlineStr">
+        <is>
+          <t>Top Preis</t>
+        </is>
+      </c>
+      <c r="O65" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="P65" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="Q65" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="R65" s="2" t="inlineStr">
+        <is>
+          <t>Mühldorf</t>
+        </is>
+      </c>
+      <c r="S65" s="2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="T65" s="2" t="inlineStr"/>
+      <c r="U65" s="2" t="inlineStr"/>
+      <c r="V65" s="2" t="inlineStr">
+        <is>
+          <t>https://www.autoscout24.de/angebote/lexus-nx-300-300h-e-four-launch-edition-elektro-benzin-silber-cat_ma43mo20491-16e8bebc-10e3-4213-9750-c0fcb2f733dd</t>
+        </is>
+      </c>
+      <c r="W65" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 09:54</t>
+        </is>
+      </c>
+      <c r="X65" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 09:54</t>
+        </is>
+      </c>
+      <c r="Y65" s="2" t="inlineStr">
+        <is>
+          <t>جدید</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="40" customHeight="1">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>AutoScout24</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Lexus RX</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>RX 450h</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>RX450H E-four Privilege !! Vermittlungsverkauf !!</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>02/2019</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>276.930 km</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>Grau</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>Elektro/Benzin</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>Automatik</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="n">
+        <v>26977</v>
+      </c>
+      <c r="L66" s="2" t="inlineStr"/>
+      <c r="M66" s="2" t="inlineStr"/>
+      <c r="N66" s="2" t="inlineStr"/>
+      <c r="O66" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="P66" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="Q66" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="R66" s="2" t="inlineStr">
+        <is>
+          <t>Micheldorf</t>
+        </is>
+      </c>
+      <c r="S66" s="2" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="T66" s="2" t="inlineStr"/>
+      <c r="U66" s="2" t="inlineStr"/>
+      <c r="V66" s="2" t="inlineStr">
+        <is>
+          <t>https://www.autoscout24.de/angebote/lexus-rx-450h-rx450h-e-four-privilege-vermittlungsverkauf-elektro-benzin-grau-cat_ma43mo19238-4a0bba83-e96f-44a2-b849-98104ed4fc2b</t>
+        </is>
+      </c>
+      <c r="W66" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 09:54</t>
+        </is>
+      </c>
+      <c r="X66" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 09:54</t>
+        </is>
+      </c>
+      <c r="Y66" s="2" t="inlineStr">
+        <is>
+          <t>جدید</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="40" customHeight="1">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>AutoScout24</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Lexus NX</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>NX 300h</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>E-Four Executive LED Navi Panorama AHK</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>02/2020</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>74.998 km</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>Rot</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>Elektro/Benzin</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>Automatik</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="n">
+        <v>29990</v>
+      </c>
+      <c r="L67" s="2" t="inlineStr"/>
+      <c r="M67" s="2" t="inlineStr"/>
+      <c r="N67" s="2" t="inlineStr">
+        <is>
+          <t>Top Preis</t>
+        </is>
+      </c>
+      <c r="O67" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="P67" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="Q67" s="2" t="inlineStr"/>
+      <c r="R67" s="2" t="inlineStr">
+        <is>
+          <t>Dresden</t>
+        </is>
+      </c>
+      <c r="S67" s="2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="T67" s="2" t="inlineStr"/>
+      <c r="U67" s="2" t="inlineStr"/>
+      <c r="V67" s="2" t="inlineStr">
+        <is>
+          <t>https://www.autoscout24.de/angebote/lexus-nx-300h-e-four-executive-led-navi-panorama-ahk-elektro-benzin-rot-cat_ma43mo75908-f3e82f16-009f-413c-892a-334e46ba7346</t>
+        </is>
+      </c>
+      <c r="W67" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 09:54</t>
+        </is>
+      </c>
+      <c r="X67" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 09:54</t>
+        </is>
+      </c>
+      <c r="Y67" s="2" t="inlineStr">
         <is>
           <t>جدید</t>
         </is>

</xml_diff>